<commit_message>
Fix type-check errors, exclude prototype sub-projects from tsconfig/jest, fix stale pre-V8 tests, fix lightweight-charts/next-auth Jest mocking, fix build script for Windows
</commit_message>
<xml_diff>
--- a/monolith-to-microservice-architecture-uionly-stack-a-b-c/microservice-architecture/microservice-architecture-update-02022026.xlsx
+++ b/monolith-to-microservice-architecture-uionly-stack-a-b-c/microservice-architecture/microservice-architecture-update-02022026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SaaS Project\trading-alerts-saas-public\monolith-to-microservice-architecture-uionly-stack-a-b-c\microservice-architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77B1BCD0-28BB-48FA-A0EA-82F94E3E28B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DE03B5-2B88-42BB-98E3-4B72E17DA1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1139" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="256">
   <si>
     <t>Part</t>
   </si>
@@ -877,48 +877,34 @@
     <t>Authentication - Backend Stack</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Mql5 (EA)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> for market data fetching from MT5 terminals + </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Python Stacks</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> for Retry/Recover/Resend machanism</t>
-    </r>
+    <t>Notifications &amp; Real-time</t>
+  </si>
+  <si>
+    <t>v2_29_data_pipeline_architecture</t>
+  </si>
+  <si>
+    <t>v2_29_multi-timeframe-visualisation</t>
+  </si>
+  <si>
+    <t>drawing-engine-line-alerts</t>
+  </si>
+  <si>
+    <t>Next.js V14 is refactored to Nest.js V11</t>
+  </si>
+  <si>
+    <t>79 fields, centroid-regression/EDT schema</t>
+  </si>
+  <si>
+    <t>Prisma Schema in Contabo VPS + SQLite in Contabo VPS</t>
+  </si>
+  <si>
+    <t>Prisma Schema : market_data_v6</t>
+  </si>
+  <si>
+    <t>Database Stack</t>
+  </si>
+  <si>
+    <t>Next.js V15.5.7 is refactored to Nest.js V11</t>
   </si>
 </sst>
 </file>
@@ -1360,7 +1346,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1671,13 +1657,34 @@
     <xf numFmtId="0" fontId="27" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6412,7 +6419,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D501F09-0F51-4028-AA61-070B2DDA5F82}">
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="2" max="2" width="28.3984375" customWidth="1"/>
@@ -6640,7 +6647,7 @@
       <c r="P11" s="9"/>
       <c r="Q11" s="10"/>
     </row>
-    <row r="12" spans="1:17" s="11" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:17" s="11" customFormat="1" ht="56.7" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A12" s="7" t="s">
         <v>7</v>
       </c>
@@ -6661,16 +6668,16 @@
         <v>7</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>228</v>
+        <v>253</v>
       </c>
       <c r="I12" s="73" t="s">
-        <v>222</v>
+        <v>254</v>
       </c>
       <c r="J12" s="43" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>146</v>
+        <v>252</v>
       </c>
       <c r="L12" s="32"/>
       <c r="M12" s="19" t="s">
@@ -6763,7 +6770,7 @@
         <v>222</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>238</v>
+        <v>255</v>
       </c>
       <c r="K14" s="9" t="s">
         <v>126</v>
@@ -6880,19 +6887,19 @@
         <v>234</v>
       </c>
       <c r="F17" s="39"/>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="116" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="I17" s="73" t="s">
+      <c r="I17" s="115" t="s">
         <v>222</v>
       </c>
-      <c r="J17" s="43" t="s">
+      <c r="J17" s="45" t="s">
         <v>234</v>
       </c>
-      <c r="K17" s="9" t="s">
+      <c r="K17" s="45" t="s">
         <v>126</v>
       </c>
       <c r="L17" s="33"/>
@@ -6939,7 +6946,7 @@
         <v>222</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="K18" s="9" t="s">
         <v>126</v>
@@ -6988,7 +6995,7 @@
         <v>222</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="K19" s="9" t="s">
         <v>126</v>
@@ -7037,7 +7044,7 @@
         <v>222</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="K20" s="9" t="s">
         <v>126</v>
@@ -7086,7 +7093,7 @@
         <v>222</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="K21" s="9" t="s">
         <v>126</v>
@@ -7135,7 +7142,7 @@
         <v>222</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="K22" s="9" t="s">
         <v>126</v>
@@ -7174,19 +7181,19 @@
         <v>233</v>
       </c>
       <c r="F23" s="39"/>
-      <c r="G23" s="14" t="s">
+      <c r="G23" s="117" t="s">
         <v>27</v>
       </c>
-      <c r="H23" s="13" t="s">
+      <c r="H23" s="82" t="s">
         <v>28</v>
       </c>
-      <c r="I23" s="73" t="s">
+      <c r="I23" s="114" t="s">
         <v>222</v>
       </c>
-      <c r="J23" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="K23" s="9" t="s">
+      <c r="J23" s="43" t="s">
+        <v>250</v>
+      </c>
+      <c r="K23" s="43" t="s">
         <v>126</v>
       </c>
       <c r="L23" s="33"/>
@@ -7233,7 +7240,7 @@
         <v>222</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="K24" s="9" t="s">
         <v>126</v>
@@ -7282,7 +7289,7 @@
         <v>222</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="K25" s="9" t="s">
         <v>126</v>
@@ -7309,7 +7316,7 @@
         <v>34</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>113</v>
+        <v>246</v>
       </c>
       <c r="C26" s="73" t="s">
         <v>97</v>
@@ -7325,13 +7332,13 @@
         <v>34</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>113</v>
+        <v>246</v>
       </c>
       <c r="I26" s="73" t="s">
         <v>222</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="K26" s="9" t="s">
         <v>126</v>
@@ -7380,7 +7387,7 @@
         <v>222</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="K27" s="9" t="s">
         <v>126</v>
@@ -7419,19 +7426,19 @@
         <v>233</v>
       </c>
       <c r="F28" s="39"/>
-      <c r="G28" s="114" t="s">
+      <c r="G28" s="118" t="s">
         <v>60</v>
       </c>
-      <c r="H28" s="115" t="s">
+      <c r="H28" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="I28" s="116" t="s">
+      <c r="I28" s="114" t="s">
         <v>222</v>
       </c>
-      <c r="J28" s="115" t="s">
-        <v>238</v>
-      </c>
-      <c r="K28" s="115" t="s">
+      <c r="J28" s="43" t="s">
+        <v>250</v>
+      </c>
+      <c r="K28" s="43" t="s">
         <v>126</v>
       </c>
       <c r="L28" s="33"/>
@@ -7468,19 +7475,19 @@
         <v>233</v>
       </c>
       <c r="F29" s="39"/>
-      <c r="G29" s="114" t="s">
+      <c r="G29" s="118" t="s">
         <v>62</v>
       </c>
-      <c r="H29" s="115" t="s">
+      <c r="H29" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="I29" s="116" t="s">
+      <c r="I29" s="114" t="s">
         <v>222</v>
       </c>
-      <c r="J29" s="115" t="s">
-        <v>238</v>
-      </c>
-      <c r="K29" s="115" t="s">
+      <c r="J29" s="43" t="s">
+        <v>250</v>
+      </c>
+      <c r="K29" s="43" t="s">
         <v>126</v>
       </c>
       <c r="L29" s="33"/>
@@ -7515,19 +7522,19 @@
         <v>233</v>
       </c>
       <c r="F30" s="39"/>
-      <c r="G30" s="114" t="s">
+      <c r="G30" s="118" t="s">
         <v>38</v>
       </c>
-      <c r="H30" s="115" t="s">
+      <c r="H30" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="I30" s="116" t="s">
+      <c r="I30" s="114" t="s">
         <v>222</v>
       </c>
-      <c r="J30" s="115" t="s">
-        <v>238</v>
-      </c>
-      <c r="K30" s="115" t="s">
+      <c r="J30" s="43" t="s">
+        <v>250</v>
+      </c>
+      <c r="K30" s="43" t="s">
         <v>126</v>
       </c>
       <c r="L30" s="33"/>
@@ -7564,19 +7571,19 @@
         <v>233</v>
       </c>
       <c r="F31" s="39"/>
-      <c r="G31" s="114" t="s">
+      <c r="G31" s="118" t="s">
         <v>76</v>
       </c>
-      <c r="H31" s="115" t="s">
+      <c r="H31" s="43" t="s">
         <v>77</v>
       </c>
-      <c r="I31" s="116" t="s">
+      <c r="I31" s="114" t="s">
         <v>222</v>
       </c>
-      <c r="J31" s="115" t="s">
-        <v>238</v>
-      </c>
-      <c r="K31" s="115" t="s">
+      <c r="J31" s="43" t="s">
+        <v>250</v>
+      </c>
+      <c r="K31" s="43" t="s">
         <v>126</v>
       </c>
       <c r="L31" s="33"/>
@@ -7596,118 +7603,144 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:17" s="11" customFormat="1" ht="27.3" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A32" s="108"/>
-      <c r="B32" s="109"/>
-      <c r="C32" s="109"/>
-      <c r="D32" s="109"/>
-      <c r="E32" s="109"/>
+    <row r="32" spans="1:17" s="11" customFormat="1" ht="27.9" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A32" s="110"/>
+      <c r="B32" s="111"/>
+      <c r="C32" s="123"/>
+      <c r="D32" s="110"/>
+      <c r="E32" s="110"/>
       <c r="F32" s="106"/>
-      <c r="G32" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="H32" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="I32" s="80" t="s">
-        <v>84</v>
-      </c>
-      <c r="J32" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="K32" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="L32" s="12"/>
-      <c r="Q32" s="18"/>
-    </row>
-    <row r="33" spans="1:17" s="11" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="G32" s="14"/>
+      <c r="H32" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="I32" s="77" t="s">
+        <v>223</v>
+      </c>
+      <c r="J32" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="K32" s="83" t="s">
+        <v>128</v>
+      </c>
+      <c r="L32" s="120"/>
+      <c r="M32" s="121"/>
+      <c r="N32" s="119"/>
+      <c r="O32" s="119"/>
+      <c r="P32" s="119"/>
+      <c r="Q32" s="122"/>
+    </row>
+    <row r="33" spans="1:17" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A33" s="108"/>
       <c r="B33" s="109"/>
       <c r="C33" s="109"/>
       <c r="D33" s="109"/>
       <c r="E33" s="109"/>
-      <c r="F33" s="107"/>
-      <c r="G33" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="H33" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="I33" s="78" t="s">
-        <v>86</v>
-      </c>
-      <c r="J33" s="9" t="s">
-        <v>246</v>
-      </c>
+      <c r="F33" s="106"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="I33" s="80"/>
+      <c r="J33" s="9"/>
       <c r="K33" s="9" t="s">
         <v>127</v>
       </c>
       <c r="L33" s="12"/>
       <c r="Q33" s="18"/>
     </row>
-    <row r="34" spans="1:17" s="11" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A34" s="51"/>
-      <c r="B34" s="52"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="42"/>
-      <c r="G34" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="H34" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="I34" s="77" t="s">
-        <v>223</v>
-      </c>
-      <c r="J34" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K34" s="83" t="s">
-        <v>128</v>
+    <row r="34" spans="1:17" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A34" s="108"/>
+      <c r="B34" s="109"/>
+      <c r="C34" s="109"/>
+      <c r="D34" s="109"/>
+      <c r="E34" s="109"/>
+      <c r="F34" s="106"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="80"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="L34" s="12"/>
       <c r="Q34" s="18"/>
     </row>
-    <row r="35" spans="1:17" s="11" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A35" s="51"/>
-      <c r="B35" s="52"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="110"/>
-      <c r="H35" s="111"/>
-      <c r="I35" s="113"/>
-      <c r="J35" s="111"/>
-      <c r="K35" s="112"/>
+    <row r="35" spans="1:17" s="11" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A35" s="108"/>
+      <c r="B35" s="109"/>
+      <c r="C35" s="109"/>
+      <c r="D35" s="109"/>
+      <c r="E35" s="109"/>
+      <c r="F35" s="107"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="I35" s="78"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9" t="s">
+        <v>127</v>
+      </c>
       <c r="L35" s="12"/>
       <c r="Q35" s="18"/>
     </row>
-    <row r="36" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A36" s="54" t="s">
+    <row r="36" spans="1:17" s="11" customFormat="1" ht="21.9" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A36" s="51"/>
+      <c r="B36" s="52"/>
+      <c r="C36" s="52"/>
+      <c r="D36" s="52"/>
+      <c r="E36" s="52"/>
+      <c r="F36" s="42"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="I36" s="77"/>
+      <c r="J36" s="13"/>
+      <c r="K36" s="83" t="s">
+        <v>126</v>
+      </c>
+      <c r="L36" s="12"/>
+      <c r="Q36" s="18"/>
+    </row>
+    <row r="37" spans="1:17" s="11" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A37" s="51"/>
+      <c r="B37" s="52"/>
+      <c r="C37" s="52"/>
+      <c r="D37" s="52"/>
+      <c r="E37" s="52"/>
+      <c r="F37" s="52"/>
+      <c r="G37" s="110"/>
+      <c r="H37" s="111"/>
+      <c r="I37" s="113"/>
+      <c r="J37" s="111"/>
+      <c r="K37" s="112"/>
+      <c r="L37" s="12"/>
+      <c r="Q37" s="18"/>
+    </row>
+    <row r="38" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A38" s="54" t="s">
         <v>243</v>
       </c>
-      <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="11"/>
-      <c r="K36" s="11"/>
-      <c r="L36" s="11"/>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.6">
-      <c r="A37" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.6">
-      <c r="A38" t="s">
-        <v>226</v>
-      </c>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
+      <c r="J38" s="11"/>
+      <c r="K38" s="11"/>
+      <c r="L38" s="11"/>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.6">
       <c r="A39" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.6">
+      <c r="A40" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.6">
+      <c r="A41" t="s">
         <v>227</v>
       </c>
     </row>
@@ -7723,6 +7756,9 @@
     <mergeCell ref="E15:E16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
+  <pageSetup scale="96" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
+  <colBreaks count="1" manualBreakCount="1">
+    <brk id="6" max="40" man="1"/>
+  </colBreaks>
 </worksheet>
 </file>
</xml_diff>